<commit_message>
new update added, this part is to treat known errors
</commit_message>
<xml_diff>
--- a/Map Opeperation/Relatorio_61.xlsx
+++ b/Map Opeperation/Relatorio_61.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\Volume Accuracy\VA\Map Opeperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A41DDBA3-E6BF-4F49-BF54-536FF5E07705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF43FFC-18C4-48CB-AE50-5C938A2988C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="61423" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="43">
   <si>
     <t>multivalues</t>
   </si>
@@ -139,6 +139,30 @@
   </si>
   <si>
     <t>363CMB(GA)+,PC(C513)-includedexcluded</t>
+  </si>
+  <si>
+    <t>CC(2.2)+,CMB(DS)+</t>
+  </si>
+  <si>
+    <t>291CC(2.2)+,CMB(DS)+includedexcluded</t>
+  </si>
+  <si>
+    <t>291</t>
+  </si>
+  <si>
+    <t>520866670</t>
+  </si>
+  <si>
+    <t>CC(2.2)+</t>
+  </si>
+  <si>
+    <t>226CC(2.2)+includedexcluded</t>
+  </si>
+  <si>
+    <t>226</t>
+  </si>
+  <si>
+    <t>522335250</t>
   </si>
 </sst>
 </file>
@@ -201,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -210,6 +234,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,7 +631,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45.453125" style="4" bestFit="1" customWidth="1"/>
@@ -834,17 +859,63 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B11" s="3"/>
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C16" s="3"/>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added a new branch for the new parten
</commit_message>
<xml_diff>
--- a/Map Opeperation/Relatorio_61.xlsx
+++ b/Map Opeperation/Relatorio_61.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\Volume Accuracy\VA\Map Opeperation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\Volume_Accuracy\Map Opeperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF43FFC-18C4-48CB-AE50-5C938A2988C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4279295F-A0B1-4C91-A399-51C2819AFA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="61423" sheetId="1" r:id="rId1"/>
-    <sheet name="61" sheetId="2" r:id="rId2"/>
+    <sheet name="61" sheetId="2" r:id="rId1"/>
+    <sheet name="61423" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -536,6 +536,303 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37849E16-F832-4CB8-B2A2-B22A8100EFE7}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="45.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.26953125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" style="4" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="4">
+        <v>358</v>
+      </c>
+      <c r="D2" s="5">
+        <v>522253720</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>341</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1002848150</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2">
+        <v>598</v>
+      </c>
+      <c r="D4" s="2">
+        <v>463555480</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2">
+        <v>598</v>
+      </c>
+      <c r="D5" s="2">
+        <v>609730010</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="4">
+        <v>358</v>
+      </c>
+      <c r="D6" s="4">
+        <v>522345300</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="4">
+        <v>363</v>
+      </c>
+      <c r="D7" s="4">
+        <v>522345300</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C14" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -626,303 +923,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37849E16-F832-4CB8-B2A2-B22A8100EFE7}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="45.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53.26953125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" style="4" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="4">
-        <v>358</v>
-      </c>
-      <c r="D2" s="5">
-        <v>522253720</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>341</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1002848150</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2">
-        <v>598</v>
-      </c>
-      <c r="D4" s="2">
-        <v>463555480</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2">
-        <v>598</v>
-      </c>
-      <c r="D5" s="2">
-        <v>609730010</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="4">
-        <v>358</v>
-      </c>
-      <c r="D6" s="4">
-        <v>522345300</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="4">
-        <v>363</v>
-      </c>
-      <c r="D7" s="4">
-        <v>522345300</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C14" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{736915f3-2f02-4945-8997-f2963298db46}" enabled="1" method="Standard" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" contentBits="1" removed="0"/>

</xml_diff>

<commit_message>
some values for single  included or excluded where failling due to float conversion, removing 00 or adding .0 to the numerico packets, this is corrected only for the normak 61 processing
</commit_message>
<xml_diff>
--- a/Map Opeperation/Relatorio_61.xlsx
+++ b/Map Opeperation/Relatorio_61.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\Volume_Accuracy\Map Opeperation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adale\OneDrive\Área de Trabalho\WESLEY- CALCULO DE VOLUMES\VA março\Map Opeperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4279295F-A0B1-4C91-A399-51C2819AFA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB876A8C-94A9-4AAA-97B1-2283953C6A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
   <si>
     <t>multivalues</t>
   </si>
@@ -63,106 +63,52 @@
     <t>FIASA</t>
   </si>
   <si>
-    <t>341MY(26)+29,39297</t>
-  </si>
-  <si>
-    <t>341</t>
-  </si>
-  <si>
-    <t>CC(1.3)+,CMB(GA)+,ECO(PL8)+,PC(C513)+</t>
-  </si>
-  <si>
-    <t>358CC(1.3)+,CMB(GA)+,ECO(PL8)+,PC(C513)+includedexcluded</t>
-  </si>
-  <si>
-    <t>097</t>
-  </si>
-  <si>
-    <t>029,392</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>MY(26)+</t>
-  </si>
-  <si>
-    <t>CMB(DS)-,TT(4X4)+</t>
-  </si>
-  <si>
-    <t>598CMB(DS)-,TT(4X4)+includedexcluded</t>
-  </si>
-  <si>
     <t>FIAPE</t>
   </si>
   <si>
     <t>RDG</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>AM(11)+</t>
   </si>
   <si>
     <t>598AM(11)+RDGexcluded</t>
   </si>
   <si>
-    <t>CMB(GA)+,MY(26)+,PC(CA79)+</t>
-  </si>
-  <si>
-    <t>358CMB(GA)+,MY(26)+,PC(CA79)+includedexcluded</t>
-  </si>
-  <si>
-    <t>A/T(TRB)+,CMB(BZ)+</t>
-  </si>
-  <si>
-    <t>363A/T(TRB)+,CMB(BZ)+includedexcluded</t>
-  </si>
-  <si>
-    <t>341MY(26)+029,097,392excluded</t>
-  </si>
-  <si>
-    <t>1002848160</t>
-  </si>
-  <si>
-    <t>029,097,392</t>
-  </si>
-  <si>
-    <t>522345300</t>
-  </si>
-  <si>
-    <t>363</t>
-  </si>
-  <si>
-    <t>CMB(GA)+,PC(C513)-</t>
-  </si>
-  <si>
-    <t>363CMB(GA)+,PC(C513)-includedexcluded</t>
-  </si>
-  <si>
-    <t>CC(2.2)+,CMB(DS)+</t>
-  </si>
-  <si>
-    <t>291CC(2.2)+,CMB(DS)+includedexcluded</t>
-  </si>
-  <si>
-    <t>291</t>
-  </si>
-  <si>
-    <t>520866670</t>
-  </si>
-  <si>
-    <t>CC(2.2)+</t>
-  </si>
-  <si>
-    <t>226CC(2.2)+includedexcluded</t>
-  </si>
-  <si>
-    <t>226</t>
-  </si>
-  <si>
-    <t>522335250</t>
+    <t>nidElementTypeParent</t>
+  </si>
+  <si>
+    <t>CMB(ALC,GA)+</t>
+  </si>
+  <si>
+    <t>FAASA</t>
+  </si>
+  <si>
+    <t>CMB(ALC)+</t>
+  </si>
+  <si>
+    <t>359CMB(ALC)+includedexcluded</t>
+  </si>
+  <si>
+    <t>CMB(ALC,GA)+,PC(CA79)+</t>
+  </si>
+  <si>
+    <t>359CMB(ALC,GA)+,PC(CA79)+includedexcluded</t>
+  </si>
+  <si>
+    <t>359CMB(ALC,GA)+includedexcluded</t>
+  </si>
+  <si>
+    <t>CMB(ALC,GA)+,PC(C513)+</t>
+  </si>
+  <si>
+    <t>359CMB(ALC,GA)+,PC(C513)+includedexcluded</t>
+  </si>
+  <si>
+    <t>358CMB(ALC)+includedexcluded</t>
   </si>
 </sst>
 </file>
@@ -225,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -233,8 +179,6 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -540,292 +484,159 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="45.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53.26953125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="4">
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2">
+        <v>359</v>
+      </c>
+      <c r="D2">
+        <v>522391460</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>359</v>
+      </c>
+      <c r="D3">
+        <v>522229500</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>359</v>
+      </c>
+      <c r="D4">
+        <v>465376850</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>359</v>
+      </c>
+      <c r="D5">
+        <v>519840640</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
         <v>358</v>
       </c>
-      <c r="D2" s="5">
-        <v>522253720</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="D6">
+        <v>522391460</v>
+      </c>
+      <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>341</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1002848150</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2">
-        <v>598</v>
-      </c>
-      <c r="D4" s="2">
-        <v>463555480</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2">
-        <v>598</v>
-      </c>
-      <c r="D5" s="2">
-        <v>609730010</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="4">
-        <v>358</v>
-      </c>
-      <c r="D6" s="4">
-        <v>522345300</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="4">
-        <v>363</v>
-      </c>
-      <c r="D7" s="4">
-        <v>522345300</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="C14" s="3"/>
-    </row>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -877,10 +688,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2">
         <v>598</v>
@@ -889,13 +700,13 @@
         <v>609730010</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H2" s="2">
         <v>1</v>
@@ -923,8 +734,274 @@
 </worksheet>
 </file>
 
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e13b492c-44e0-478c-a27b-4b735264ccb7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1096d648-6e9c-4990-8f73-aa0f2ab1a217">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA1DFDF4B147C34BB45DD9C94654ACC2" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="897bd39cf1d1b4d81f36a51d3a3e06a6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1096d648-6e9c-4990-8f73-aa0f2ab1a217" xmlns:ns3="e13b492c-44e0-478c-a27b-4b735264ccb7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6707c27936323c15de64aa66c05905b8" ns2:_="" ns3:_="">
+    <xsd:import namespace="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+    <xsd:import namespace="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1096d648-6e9c-4990-8f73-aa0f2ab1a217" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="9247bebf-ce0e-4fa1-bae7-748a1283d6fa" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="18" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="19" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e13b492c-44e0-478c-a27b-4b735264ccb7" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{a993a088-c5ed-4b9a-9cf0-e9a75d274e9d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e13b492c-44e0-478c-a27b-4b735264ccb7">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C109B92B-4E8D-418B-8D81-805584D1A006}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <ds:schemaRef ds:uri="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5BB71BB-4640-40BB-8D40-ADCD285100FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1096d648-6e9c-4990-8f73-aa0f2ab1a217"/>
+    <ds:schemaRef ds:uri="e13b492c-44e0-478c-a27b-4b735264ccb7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD988340-D21F-415F-9B37-7D4F54448A31}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{725ca717-11da-4935-b601-f527b9741f2e}" enabled="1" method="Standard" siteId="{d852d5cd-724c-4128-8812-ffa5db3f8507}" contentBits="0" removed="0"/>
   <clbl:label id="{736915f3-2f02-4945-8997-f2963298db46}" enabled="1" method="Standard" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" contentBits="1" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>